<commit_message>
we zijn er bijna
</commit_message>
<xml_diff>
--- a/eerstejaarsquiz_template_alw.xlsx
+++ b/eerstejaarsquiz_template_alw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thomasvanhoey/Library/CloudStorage/Dropbox/1_Projects_ongoing/lingquiztics/quiz_europese_taalkunde_2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D6A8FAB3-1441-034A-A4B5-0C509576D1D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BDB0486-BB8F-F44C-9D31-98D7A1284731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="33740" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="33740" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template (Rondenaam) " sheetId="6" r:id="rId1"/>
@@ -22,7 +22,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ALW Random'!$A$1:$K$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Template (ALW Cryptogramm)  '!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Template (ALW Cryptogramm)  '!$A$1:$J$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Template (Literatuur in kunst)'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Template (Literatuur-memes)'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Template (Oulipo S+7) '!$A$1:$K$1</definedName>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="207">
   <si>
     <t>description</t>
   </si>
@@ -1332,24 +1332,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12E914F5-CE0D-4364-9E80-368BD71E139F}">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.83203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="26.6640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.6640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="29" style="1" customWidth="1"/>
-    <col min="5" max="5" width="21.6640625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="18.33203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="19.6640625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="25" style="1" customWidth="1"/>
-    <col min="10" max="10" width="15" style="1" customWidth="1"/>
-    <col min="11" max="11" width="25.33203125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="18.1640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="30.83203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="19.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="25" style="1" customWidth="1"/>
+    <col min="9" max="9" width="15" style="1" customWidth="1"/>
+    <col min="10" max="10" width="25.33203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="18.1640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="30" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="30" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1360,31 +1359,28 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="64" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>174</v>
       </c>
@@ -1394,88 +1390,88 @@
       <c r="C2" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="B3" s="6" t="s">
         <v>178</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="B4" s="6" t="s">
         <v>181</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="B5" s="6" t="s">
         <v>184</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="B6" s="6" t="s">
         <v>187</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>190</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="B8" s="5" t="s">
         <v>193</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="B9" s="6" t="s">
         <v>196</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="B10" s="6" t="s">
         <v>199</v>
       </c>
@@ -1483,7 +1479,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="B11" s="6" t="s">
         <v>201</v>
       </c>
@@ -1492,7 +1488,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:J1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>